<commit_message>
Fix Excel subnet calculator: real binary view, mask input, validation
- Binary View (B23:B25) uses DEC2BIN(octet,8) instead of zero-padded decimal
- Optional Subnet Mask (B7) now drives the prefix when it is a valid mask
  (1-bit lookup per octet + contiguity check); falls back to CIDR in B6
- B6 data validation now shows its error (whole number 0-32)
- Red status notes for invalid IP (C5) and invalid mask (C7)
- Instructions: drop BITAND/BITOR claim; works as-is in Excel/LibreOffice/Sheets
- Python Script sheet: no full host list, unused imports removed, IPv4-only check
- Re-rendered screenshot
</commit_message>
<xml_diff>
--- a/excel-subnet-calculator/IPv4_Subnet_Calculator.xlsx
+++ b/excel-subnet-calculator/IPv4_Subnet_Calculator.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Python Script" sheetId="2" r:id="rId2"/>
     <sheet name="Instructions" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191028" iterateDelta="1E-4"/>
+  <calcPr calcId="191028" fullCalcOnLoad="1" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
   <si>
     <t>IPv4 Subnet Calculator</t>
   </si>
@@ -233,9 +233,9 @@
     <t>Companion Python Script (ipaddress module)</t>
   </si>
   <si>
-    <t># Save this as subnet_calc.py and run with:  python subnet_calc.py
+    <t xml:space="preserve"># Save this as subnet_calc.py and run with:  python subnet_calc.py
 # Requires Python 3.3+ (ipaddress is in the standard library)
-from ipaddress import ip_network, ip_interface, IPv4Network
+from ipaddress import IPv4Network, ip_network
 import sys
 def calculate_subnet(cidr: str):
     """Calculate and print full subnet details for an IPv4 CIDR."""
@@ -244,6 +244,9 @@
         net = ip_network(cidr, strict=False)  # strict=False allows host bits set
     except ValueError as e:
         print(f"Invalid input: {e}")
+        return
+    if not isinstance(net, IPv4Network):
+        print(f"Invalid input: {cidr!r} is not an IPv4 network (this calculator is IPv4 only)")
         return
     print("=" * 50)
     print(f"Input CIDR          : {cidr}")
@@ -262,10 +265,10 @@
         usable = 1
         first = last = net.network_address
     else:
+        # Simple math instead of building the whole host list (fast even for a /8)
         usable = net.num_addresses - 2
-        hosts = list(net.hosts())
-        first = hosts[0] if hosts else None
-        last = hosts[-1] if hosts else None
+        first = net.network_address + 1
+        last = net.broadcast_address - 1
     print(f"Usable Hosts        : {usable}")
     print(f"First Usable Host   : {first}")
     print(f"Last Usable Host    : {last}")
@@ -319,10 +322,10 @@
     <t>6. Green cells are calculated – do not type over them.</t>
   </si>
   <si>
-    <t>Requirements: Excel 2013 or later / Microsoft 365 (BITAND and BITOR functions).</t>
-  </si>
-  <si>
-    <t>Works in Google Sheets with minor adjustments (BITAND/BITOR are available).</t>
+    <t xml:space="preserve">Requirements: none beyond standard formulas (FIND, MID, VALUE, INT, MOD, MATCH, DEC2BIN). No macros or add-ins.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Works as-is in Microsoft Excel, LibreOffice Calc and Google Sheets.</t>
   </si>
   <si>
     <t>SHEET 2 – Python Script</t>
@@ -563,7 +566,14 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFC00000"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -876,8 +886,9 @@
       <c r="B5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="7" t="s">
-        <v>7</v>
+      <c r="C5" s="7" t="str">
+        <f>IF(M6,"← Edit this (blue text = input)","⚠ Invalid IP: need 4 octets, each 0-255")</f>
+        <v>← Edit this (blue text = input)</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>8</v>
@@ -909,7 +920,7 @@
         <v>168427789</v>
       </c>
       <c r="M5">
-        <f>B6</f>
+        <f>IF(M7,M8,B6)</f>
         <v>18</v>
       </c>
     </row>
@@ -952,14 +963,19 @@
         <f>H6*16777216+I6*65536+J6*256+K6</f>
         <v>4294950912</v>
       </c>
+      <c r="M6" t="b">
+        <f>IFERROR(AND(H5&amp;"."&amp;I5&amp;"."&amp;J5&amp;"."&amp;K5=TRIM(B5),MAX(H5:K5)&lt;=255,MIN(H5:K5)&gt;=0),FALSE)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1">
       <c r="A7" s="5" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="6"/>
-      <c r="C7" s="7" t="s">
-        <v>17</v>
+      <c r="C7" s="7" t="str">
+        <f>IF(TRIM(B7)="","Leave blank to use CIDR only",IF(M7,"✓ Mask in use: /"&amp;M8&amp;" (overrides B6)","⚠ Invalid mask: using CIDR in B6"))</f>
+        <v>Leave blank to use CIDR only</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>18</v>
@@ -974,6 +990,10 @@
         <f>INT(L5/(2^(32-M5)))*(2^(32-M5))</f>
         <v>168427520</v>
       </c>
+      <c r="M7" t="b">
+        <f>IFERROR(AND(H9&amp;"."&amp;I9&amp;"."&amp;J9&amp;"."&amp;K9=TRIM(B7),MIN(H10:K10)&gt;=0,OR(I9=0,H9=255),OR(J9=0,I9=255),OR(K9=0,J9=255)),FALSE)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1">
       <c r="D8" s="9" t="s">
@@ -1005,6 +1025,10 @@
         <f>H8*16777216+I8*65536+J8*256+K8</f>
         <v>16383</v>
       </c>
+      <c r="M8">
+        <f>SUM(H10:K10)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1">
       <c r="A9" s="1" t="s">
@@ -1020,6 +1044,22 @@
       <c r="F9" s="10" t="s">
         <v>27</v>
       </c>
+      <c r="H9">
+        <f>IFERROR(VALUE(LEFT(B7,FIND(".",B7)-1)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <f>IFERROR(VALUE(MID(B7,FIND(".",B7)+1,FIND(".",B7,FIND(".",B7)+1)-FIND(".",B7)-1)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <f>IFERROR(VALUE(MID(B7,FIND(".",B7,FIND(".",B7)+1)+1,FIND(".",B7,FIND(".",B7,FIND(".",B7)+1)+1)-FIND(".",B7,FIND(".",B7)+1)-1)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <f>IFERROR(VALUE(RIGHT(B7,LEN(B7)-FIND(".",B7,FIND(".",B7,FIND(".",B7)+1)+1))),0)</f>
+        <v>0</v>
+      </c>
       <c r="L9">
         <f>L7+(2^(32-M5))-1</f>
         <v>168443903</v>
@@ -1042,6 +1082,22 @@
       <c r="F10" s="9" t="s">
         <v>31</v>
       </c>
+      <c r="H10">
+        <f>IFERROR(9-MATCH(H9,{255,254,252,248,240,224,192,128,0},0),-1)</f>
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <f>IFERROR(9-MATCH(I9,{255,254,252,248,240,224,192,128,0},0),-1)</f>
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <f>IFERROR(9-MATCH(J9,{255,254,252,248,240,224,192,128,0},0),-1)</f>
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <f>IFERROR(9-MATCH(K9,{255,254,252,248,240,224,192,128,0},0),-1)</f>
+        <v>0</v>
+      </c>
       <c r="L10">
         <f>IF(M5=32,L5,IF(M5=31,L7,L7+1))</f>
         <v>168427521</v>
@@ -1206,8 +1262,8 @@
         <v>59</v>
       </c>
       <c r="B23" s="13" t="str">
-        <f>TEXT(H5,"00000000")&amp;"."&amp;TEXT(I5,"00000000")&amp;"."&amp;TEXT(J5,"00000000")&amp;"."&amp;TEXT(K5,"00000000")</f>
-        <v>00000010.00000010.00000001.00000013</v>
+        <f>DEC2BIN(H5,8)&amp;"."&amp;DEC2BIN(I5,8)&amp;"."&amp;DEC2BIN(J5,8)&amp;"."&amp;DEC2BIN(K5,8)</f>
+        <v>00001010.00001010.00000001.00001101</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="15" customHeight="1">
@@ -1215,8 +1271,8 @@
         <v>60</v>
       </c>
       <c r="B24" s="13" t="str">
-        <f>TEXT(H6,"00000000")&amp;"."&amp;TEXT(I6,"00000000")&amp;"."&amp;TEXT(J6,"00000000")&amp;"."&amp;TEXT(K6,"00000000")</f>
-        <v>00000255.00000255.00000192.00000000</v>
+        <f>DEC2BIN(H6,8)&amp;"."&amp;DEC2BIN(I6,8)&amp;"."&amp;DEC2BIN(J6,8)&amp;"."&amp;DEC2BIN(K6,8)</f>
+        <v>11111111.11111111.11000000.00000000</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="15" customHeight="1">
@@ -1224,8 +1280,8 @@
         <v>61</v>
       </c>
       <c r="B25" s="13" t="str">
-        <f>TEXT(INT(L7/16777216),"00000000")&amp;"."&amp;TEXT(INT(MOD(L7,16777216)/65536),"00000000")&amp;"."&amp;TEXT(INT(MOD(L7,65536)/256),"00000000")&amp;"."&amp;TEXT(MOD(L7,256),"00000000")</f>
-        <v>00000010.00000010.00000000.00000000</v>
+        <f>DEC2BIN(INT(L7/16777216),8)&amp;"."&amp;DEC2BIN(INT(MOD(L7,16777216)/65536),8)&amp;"."&amp;DEC2BIN(INT(MOD(L7,65536)/256),8)&amp;"."&amp;DEC2BIN(MOD(L7,256),8)</f>
+        <v>00001010.00001010.00000000.00000000</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="15" customHeight="1">
@@ -1259,8 +1315,18 @@
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="A9:B9"/>
   </mergeCells>
+  <conditionalFormatting sqref="C5">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>NOT($M$6)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C7">
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>AND(TRIM($B$7)&lt;&gt;"",NOT($M$7))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="whole" errorTitle="Invalid CIDR" error="CIDR must be an integer between 0 and 32" sqref="B6" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Invalid CIDR" error="CIDR must be an integer between 0 and 32" sqref="B6" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>0</formula1>
       <formula2>32</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Shorter invalid-IP warning; blank binary rows for an invalid IP
- C5 warning is now "⚠ Invalid IP (each octet 0-255)" so it fits column C
- B23 (IP) and B25 (network) binary rows show "—" when the IP is invalid
  instead of #NUM!/Err:502; B24 (mask) is unchanged
- README notes the binary-row behavior
</commit_message>
<xml_diff>
--- a/excel-subnet-calculator/IPv4_Subnet_Calculator.xlsx
+++ b/excel-subnet-calculator/IPv4_Subnet_Calculator.xlsx
@@ -887,7 +887,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="7" t="str">
-        <f>IF(M6,"← Edit this (blue text = input)","⚠ Invalid IP: need 4 octets, each 0-255")</f>
+        <f>IF(M6,"← Edit this (blue text = input)","⚠ Invalid IP (each octet 0-255)")</f>
         <v>← Edit this (blue text = input)</v>
       </c>
       <c r="D5" s="8" t="s">
@@ -1262,7 +1262,7 @@
         <v>59</v>
       </c>
       <c r="B23" s="13" t="str">
-        <f>DEC2BIN(H5,8)&amp;"."&amp;DEC2BIN(I5,8)&amp;"."&amp;DEC2BIN(J5,8)&amp;"."&amp;DEC2BIN(K5,8)</f>
+        <f>IF(M6,DEC2BIN(H5,8)&amp;"."&amp;DEC2BIN(I5,8)&amp;"."&amp;DEC2BIN(J5,8)&amp;"."&amp;DEC2BIN(K5,8),"—")</f>
         <v>00001010.00001010.00000001.00001101</v>
       </c>
     </row>
@@ -1280,7 +1280,7 @@
         <v>61</v>
       </c>
       <c r="B25" s="13" t="str">
-        <f>DEC2BIN(INT(L7/16777216),8)&amp;"."&amp;DEC2BIN(INT(MOD(L7,16777216)/65536),8)&amp;"."&amp;DEC2BIN(INT(MOD(L7,65536)/256),8)&amp;"."&amp;DEC2BIN(MOD(L7,256),8)</f>
+        <f>IF(M6,DEC2BIN(INT(L7/16777216),8)&amp;"."&amp;DEC2BIN(INT(MOD(L7,16777216)/65536),8)&amp;"."&amp;DEC2BIN(INT(MOD(L7,65536)/256),8)&amp;"."&amp;DEC2BIN(MOD(L7,256),8),"—")</f>
         <v>00001010.00001010.00000000.00000000</v>
       </c>
     </row>

</xml_diff>